<commit_message>
Add postoperative creatinine timing and follow-up coverage diagnostic for v3.4.0
</commit_message>
<xml_diff>
--- a/workbook/All_Revised_Tables.xlsx
+++ b/workbook/All_Revised_Tables.xlsx
@@ -2,51 +2,56 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INDEX" sheetId="1" r:id="R2459d2239d7f4461"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_1" sheetId="2" r:id="R555492e9f0c14fe3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_2" sheetId="3" r:id="R4adbdf5abd6c4e31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_3" sheetId="4" r:id="R93a7f2b0cf4d46cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_4" sheetId="5" r:id="R28da0ea953bd4c0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S1" sheetId="6" r:id="R9bcb8182e39844a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S2" sheetId="7" r:id="R1ebcd96f28a64bf0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S3" sheetId="8" r:id="R57de617c2a004ddf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S4" sheetId="9" r:id="R516be881f7dd465b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S5" sheetId="10" r:id="Rff877797a7a547a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S6" sheetId="11" r:id="R9ae43eb372514955"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S7" sheetId="12" r:id="R302fce89dc1442ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S8" sheetId="13" r:id="R1ef7340489184ed3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S9" sheetId="14" r:id="R5c931b3ae55940d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S10" sheetId="15" r:id="R84bea2eb07874051"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S11" sheetId="16" r:id="Re92f8aa7c25e44e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S12" sheetId="17" r:id="Rf6d34a8c9b9b4d5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S13" sheetId="18" r:id="R5c9bc62681a54880"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S14" sheetId="19" r:id="R0066b9e99c1d4da8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S15" sheetId="20" r:id="R21477df62e2a49ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S16" sheetId="21" r:id="R5a4a8f28f98c46bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S17" sheetId="22" r:id="R4ed0595c576940a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S18" sheetId="23" r:id="Rb6d032b59a574c83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S19" sheetId="24" r:id="R55c04b5b1de54f81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S20" sheetId="25" r:id="Rb65ec817c26847a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S1b" sheetId="26" r:id="R78f6447aaee94de7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S21" sheetId="27" r:id="R63e790471bb84919"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S22" sheetId="28" r:id="R9833c8287c1a4cd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S23" sheetId="29" r:id="R27f8a7c2bd1a455f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S24" sheetId="30" r:id="R2f65b3bdf1404a00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S25" sheetId="31" r:id="Re3c00c046d3a4a5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S25b" sheetId="32" r:id="R788b93668d59400c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S26" sheetId="33" r:id="Rc4a0a12ef50f4194"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1_Flow_numeric" sheetId="34" r:id="Rb800d731f9df4f77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S21_numeric" sheetId="35" r:id="R63dcd6aa5967425f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S22_numeric" sheetId="36" r:id="R136197081e754b14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S23_numeric" sheetId="37" r:id="R3c2793198bbb4d64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S24_numeric" sheetId="38" r:id="R22d5997280894811"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S25_CI_numeric" sheetId="39" r:id="R00e0f42d65574e8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S25_Difference_numeric" sheetId="40" r:id="R0f695d0647454fa2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Primary_numeric" sheetId="41" r:id="Rf94954eedcd542cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparators_numeric" sheetId="42" r:id="Rd072240f98b441e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workload_numeric" sheetId="43" r:id="Rfed5783586464e3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S27" sheetId="44" r:id="R2fe0a7be1c194af4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S27_numeric" sheetId="45" r:id="R07b9146dcdcf4e6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INDEX" sheetId="1" r:id="R12e511f916114e32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_1" sheetId="2" r:id="Rb0caf84ce1a54236"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_2" sheetId="3" r:id="R6dd2e148605c4cdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_3" sheetId="4" r:id="R0cfe0ec0b70548d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_4" sheetId="5" r:id="R7cbcf67ade6944b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S1" sheetId="6" r:id="Rd36d400468194cf6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S2" sheetId="7" r:id="Rcc19447bba4641f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S3" sheetId="8" r:id="Rc233ebd39b884df9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S4" sheetId="9" r:id="R840fbe591204488d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S5" sheetId="10" r:id="R3d7f5ea706334385"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S6" sheetId="11" r:id="R181e9cfb91e14755"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S7" sheetId="12" r:id="R28e3f04f9ee34049"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S8" sheetId="13" r:id="R98a06588dde04ded"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S9" sheetId="14" r:id="Rd127e313cf044ce1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S10" sheetId="15" r:id="R6e456bc5bc5240e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S11" sheetId="16" r:id="Rd757df5cc9be4289"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S12" sheetId="17" r:id="Rdd17577656814d81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S13" sheetId="18" r:id="Rac6abfac7ac44d12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S14" sheetId="19" r:id="R076219054eba4098"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S15" sheetId="20" r:id="R72fb42c35f3443c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S16" sheetId="21" r:id="Rbf6c2e6f11bc4158"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S17" sheetId="22" r:id="Rda08f57de72d405c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S18" sheetId="23" r:id="Red1b7ae39d4446c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S19" sheetId="24" r:id="Rde908fd2e5964c10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S20" sheetId="25" r:id="Rab7d1442c2724468"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S1b" sheetId="26" r:id="R70b9c15bcee64b60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S21" sheetId="27" r:id="R7b3b2aebfb8e4054"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S22" sheetId="28" r:id="Re4391a7cdf864f1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S23" sheetId="29" r:id="R370695edf7aa483a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S24" sheetId="30" r:id="R11c10d9146ee4354"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S25" sheetId="31" r:id="R6db6d6049a694ae7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S25b" sheetId="32" r:id="R6d24372f88cc4453"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S26" sheetId="33" r:id="R8c5a052f4b4e4ea1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1_Flow_numeric" sheetId="34" r:id="R1e610a5a72214242"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S21_numeric" sheetId="35" r:id="Rc5289a76a0474cf2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S22_numeric" sheetId="36" r:id="R9ae17d57111c44c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S23_numeric" sheetId="37" r:id="R682f42eeb14e4cda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S24_numeric" sheetId="38" r:id="R252a8f0817fc4361"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S25_CI_numeric" sheetId="39" r:id="R515507b0bc434857"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S25_Difference_numeric" sheetId="40" r:id="Re147aeb5c989486b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Primary_numeric" sheetId="41" r:id="Rdefc21629e0745ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparators_numeric" sheetId="42" r:id="Rf864779e3f21458b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workload_numeric" sheetId="43" r:id="Rbd1f605c65054f70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S27" sheetId="44" r:id="R06a19e49783a4146"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S27_numeric" sheetId="45" r:id="R0e33eee958424737"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S28" sheetId="46" r:id="Ra092db984f254b2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S29" sheetId="47" r:id="Rd9afacff212f4b92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S30" sheetId="48" r:id="R5238e6cc46394516"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_S31" sheetId="49" r:id="Rda973bcd5e874d95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timing_Definitions" sheetId="50" r:id="R8dc906da5ac74f00"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -57,15 +62,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="6">
+  <x:numFmts count="7">
     <x:numFmt numFmtId="200" formatCode="#,##0"/>
     <x:numFmt numFmtId="201" formatCode="0.0000"/>
     <x:numFmt numFmtId="202" formatCode="0.0000000000"/>
     <x:numFmt numFmtId="203" formatCode="0.000000"/>
     <x:numFmt numFmtId="204" formatCode="0.00000"/>
     <x:numFmt numFmtId="205" formatCode="0.00%"/>
+    <x:numFmt numFmtId="206" formatCode="0.0"/>
   </x:numFmts>
-  <x:fonts count="9">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -112,8 +118,18 @@
       <x:sz val="10"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -143,8 +159,13 @@
         <x:fgColor rgb="FFF3F4F5"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9E4E8"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="3">
+  <x:borders count="4">
     <x:border/>
     <x:border/>
     <x:border>
@@ -152,12 +173,26 @@
         <x:color rgb="FFB4B8BD"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="2">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="4" fillId="4" borderId="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="39">
+  <x:cellXfs count="48">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -290,6 +325,31 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -878,6 +938,46 @@
         <x:v>Unrounded same-timestamp baseline-selection sensitivity outputs</x:v>
       </x:c>
     </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="47" t="str">
+        <x:v>Table_S28</x:v>
+      </x:c>
+      <x:c r="B48" s="47" t="str">
+        <x:v>Testing-time and follow-up diagnostic, 7 October 2026; included in v3.4.0; see the GitHub release for the assigned version DOI</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="47" t="str">
+        <x:v>Table_S29</x:v>
+      </x:c>
+      <x:c r="B49" s="47" t="str">
+        <x:v>Testing-time and follow-up diagnostic, 7 October 2026; included in v3.4.0; see the GitHub release for the assigned version DOI</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="47" t="str">
+        <x:v>Table_S30</x:v>
+      </x:c>
+      <x:c r="B50" s="47" t="str">
+        <x:v>Testing-time and follow-up diagnostic, 7 October 2026; included in v3.4.0; see the GitHub release for the assigned version DOI</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="47" t="str">
+        <x:v>Table_S31</x:v>
+      </x:c>
+      <x:c r="B51" s="47" t="str">
+        <x:v>Testing-time and follow-up diagnostic, 7 October 2026; included in v3.4.0; see the GitHub release for the assigned version DOI</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="47" t="str">
+        <x:v>Timing_Definitions</x:v>
+      </x:c>
+      <x:c r="B52" s="47" t="str">
+        <x:v>Testing-time and follow-up diagnostic, 7 October 2026; included in v3.4.0; see the GitHub release for the assigned version DOI</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -19089,6 +19189,2375 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="53" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="43" customHeight="1">
+      <x:c r="A1" s="44" t="str">
+        <x:v>Measure</x:v>
+      </x:c>
+      <x:c r="B1" s="44" t="str">
+        <x:v>INSPIRE</x:v>
+      </x:c>
+      <x:c r="C1" s="44" t="str">
+        <x:v>MOVER 2021</x:v>
+      </x:c>
+      <x:c r="D1" s="44" t="str">
+        <x:v>MOVER 2022</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="43" customHeight="1">
+      <x:c r="A2" s="45" t="str">
+        <x:v>Any postoperative test</x:v>
+      </x:c>
+      <x:c r="B2" s="45" t="str">
+        <x:v>24872/33394 (74.5%) [74.0-74.9]</x:v>
+      </x:c>
+      <x:c r="C2" s="45" t="str">
+        <x:v>2212/2802 (78.9%) [77.4-80.4]</x:v>
+      </x:c>
+      <x:c r="D2" s="45" t="str">
+        <x:v>2033/2587 (78.6%) [77.0-80.1]</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="43" customHeight="1">
+      <x:c r="A3" s="45" t="str">
+        <x:v>No postoperative test</x:v>
+      </x:c>
+      <x:c r="B3" s="45" t="str">
+        <x:v>8522/33394 (25.5%) [25.1-26.0]</x:v>
+      </x:c>
+      <x:c r="C3" s="45" t="str">
+        <x:v>590/2802 (21.1%) [19.6-22.6]</x:v>
+      </x:c>
+      <x:c r="D3" s="45" t="str">
+        <x:v>554/2587 (21.4%) [19.9-23.0]</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="43" customHeight="1">
+      <x:c r="A4" s="45" t="str">
+        <x:v>Test in (0,48] h</x:v>
+      </x:c>
+      <x:c r="B4" s="45" t="str">
+        <x:v>24488/33394 (73.3%) [72.9-73.8]</x:v>
+      </x:c>
+      <x:c r="C4" s="45" t="str">
+        <x:v>2194/2802 (78.3%) [76.7-79.8]</x:v>
+      </x:c>
+      <x:c r="D4" s="45" t="str">
+        <x:v>2018/2587 (78.0%) [76.4-79.6]</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="43" customHeight="1">
+      <x:c r="A5" s="45" t="str">
+        <x:v>Test in (48,168] h before recorded stop</x:v>
+      </x:c>
+      <x:c r="B5" s="45" t="str">
+        <x:v>18498/33394 (55.4%) [54.9-55.9]</x:v>
+      </x:c>
+      <x:c r="C5" s="45" t="str">
+        <x:v>1358/2802 (48.5%) [46.6-50.3]</x:v>
+      </x:c>
+      <x:c r="D5" s="45" t="str">
+        <x:v>1305/2587 (50.4%) [48.5-52.4]</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="43" customHeight="1">
+      <x:c r="A6" s="45" t="str">
+        <x:v>Tests in both early and late windows</x:v>
+      </x:c>
+      <x:c r="B6" s="45" t="str">
+        <x:v>18114/33394 (54.2%) [53.7-54.8]</x:v>
+      </x:c>
+      <x:c r="C6" s="45" t="str">
+        <x:v>1340/2802 (47.8%) [46.0-49.7]</x:v>
+      </x:c>
+      <x:c r="D6" s="45" t="str">
+        <x:v>1290/2587 (49.9%) [47.9-51.8]</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="43" customHeight="1">
+      <x:c r="A7" s="45" t="str">
+        <x:v>Only one distinct testing time</x:v>
+      </x:c>
+      <x:c r="B7" s="45" t="str">
+        <x:v>4040/33394 (12.1%) [11.8-12.5]</x:v>
+      </x:c>
+      <x:c r="C7" s="45" t="str">
+        <x:v>489/2802 (17.5%) [16.1-18.9]</x:v>
+      </x:c>
+      <x:c r="D7" s="45" t="str">
+        <x:v>405/2587 (15.7%) [14.3-17.1]</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="43" customHeight="1">
+      <x:c r="A8" s="45" t="str">
+        <x:v>Algorithmic observation window &lt;48 h</x:v>
+      </x:c>
+      <x:c r="B8" s="45" t="str">
+        <x:v>5317/33394 (15.9%) [15.5-16.3]</x:v>
+      </x:c>
+      <x:c r="C8" s="45" t="str">
+        <x:v>1162/2802 (41.5%) [39.7-43.3]</x:v>
+      </x:c>
+      <x:c r="D8" s="45" t="str">
+        <x:v>979/2587 (37.8%) [36.0-39.7]</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="43" customHeight="1">
+      <x:c r="A9" s="45" t="str">
+        <x:v>Algorithmic observation window &lt;168 h</x:v>
+      </x:c>
+      <x:c r="B9" s="45" t="str">
+        <x:v>21415/33394 (64.1%) [63.6-64.6]</x:v>
+      </x:c>
+      <x:c r="C9" s="45" t="str">
+        <x:v>2149/2802 (76.7%) [75.1-78.2]</x:v>
+      </x:c>
+      <x:c r="D9" s="45" t="str">
+        <x:v>1898/2587 (73.4%) [71.6-75.0]</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="43" customHeight="1">
+      <x:c r="A10" s="45" t="str">
+        <x:v>Discharge stop time missing or unusable</x:v>
+      </x:c>
+      <x:c r="B10" s="45" t="str">
+        <x:v>&lt;5/33394 (suppressed)</x:v>
+      </x:c>
+      <x:c r="C10" s="45" t="str">
+        <x:v>&lt;5/2802 (suppressed)</x:v>
+      </x:c>
+      <x:c r="D10" s="45" t="str">
+        <x:v>&lt;5/2587 (suppressed)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="43" customHeight="1">
+      <x:c r="A11" s="45" t="str">
+        <x:v>Early test among algorithmic window &gt;=48 h</x:v>
+      </x:c>
+      <x:c r="B11" s="45" t="str">
+        <x:v>22989/28077 (81.9%) [81.4-82.3]</x:v>
+      </x:c>
+      <x:c r="C11" s="45" t="str">
+        <x:v>1590/1640 (97.0%) [96.0-97.7]</x:v>
+      </x:c>
+      <x:c r="D11" s="45" t="str">
+        <x:v>1540/1608 (95.8%) [94.7-96.7]</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="43" customHeight="1">
+      <x:c r="A12" s="45" t="str">
+        <x:v>Late test among algorithmic window &gt;48 h</x:v>
+      </x:c>
+      <x:c r="B12" s="45" t="str">
+        <x:v>18498/28066 (65.9%) [65.4-66.5]</x:v>
+      </x:c>
+      <x:c r="C12" s="45" t="str">
+        <x:v>1358/1640 (82.8%) [80.9-84.6]</x:v>
+      </x:c>
+      <x:c r="D12" s="45" t="str">
+        <x:v>1305/1608 (81.2%) [79.2-83.0]</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="43" customHeight="1">
+      <x:c r="A13" s="45" t="str">
+        <x:v>First test hours among observed</x:v>
+      </x:c>
+      <x:c r="B13" s="45" t="str">
+        <x:v>0.6 (0.3-17.2)</x:v>
+      </x:c>
+      <x:c r="C13" s="45" t="str">
+        <x:v>12.0 (2.1-16.9)</x:v>
+      </x:c>
+      <x:c r="D13" s="45" t="str">
+        <x:v>11.9 (1.9-17.0)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="43" customHeight="1">
+      <x:c r="A14" s="45" t="str">
+        <x:v>Last test hours among observed</x:v>
+      </x:c>
+      <x:c r="B14" s="45" t="str">
+        <x:v>111.5 (46.9-156.4)</x:v>
+      </x:c>
+      <x:c r="C14" s="45" t="str">
+        <x:v>70.9 (28.7-147.6)</x:v>
+      </x:c>
+      <x:c r="D14" s="45" t="str">
+        <x:v>83.9 (35.6-153.1)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="43" customHeight="1">
+      <x:c r="A15" s="45" t="str">
+        <x:v>Testing occasions among observed</x:v>
+      </x:c>
+      <x:c r="B15" s="45" t="str">
+        <x:v>3.0 (2.0-5.0)</x:v>
+      </x:c>
+      <x:c r="C15" s="45" t="str">
+        <x:v>4.0 (2.0-7.0)</x:v>
+      </x:c>
+      <x:c r="D15" s="45" t="str">
+        <x:v>4.0 (2.0-7.0)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="43" customHeight="1">
+      <x:c r="A16" s="45" t="str">
+        <x:v>Elapsed 24 h bins with test among observed</x:v>
+      </x:c>
+      <x:c r="B16" s="45" t="str">
+        <x:v>3.0 (2.0-4.0)</x:v>
+      </x:c>
+      <x:c r="C16" s="45" t="str">
+        <x:v>3.0 (1.0-6.0)</x:v>
+      </x:c>
+      <x:c r="D16" s="45" t="str">
+        <x:v>3.0 (2.0-7.0)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="43" customHeight="1">
+      <x:c r="A17" s="45" t="str">
+        <x:v>Gap from last test to recorded stop among observed</x:v>
+      </x:c>
+      <x:c r="B17" s="45" t="str">
+        <x:v>22.2 (11.4-39.8)</x:v>
+      </x:c>
+      <x:c r="C17" s="45" t="str">
+        <x:v>9.1 (5.6-13.8)</x:v>
+      </x:c>
+      <x:c r="D17" s="45" t="str">
+        <x:v>9.7 (6.1-14.4)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="43" customHeight="1">
+      <x:c r="A18" s="45" t="str">
+        <x:v>Observation opportunity hours</x:v>
+      </x:c>
+      <x:c r="B18" s="45" t="str">
+        <x:v>127.6 (61.3-168.0)</x:v>
+      </x:c>
+      <x:c r="C18" s="45" t="str">
+        <x:v>69.7 (22.8-158.9)</x:v>
+      </x:c>
+      <x:c r="D18" s="45" t="str">
+        <x:v>73.8 (24.2-168.0)</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="20" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="20" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="20" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="20" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="20" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="72" customHeight="1">
+      <x:c r="A1" s="44" t="str">
+        <x:v>cohort</x:v>
+      </x:c>
+      <x:c r="B1" s="44" t="str">
+        <x:v>group</x:v>
+      </x:c>
+      <x:c r="C1" s="44" t="str">
+        <x:v>eligible_n</x:v>
+      </x:c>
+      <x:c r="D1" s="44" t="str">
+        <x:v>observed_n</x:v>
+      </x:c>
+      <x:c r="E1" s="44" t="str">
+        <x:v>observed_pct</x:v>
+      </x:c>
+      <x:c r="F1" s="44" t="str">
+        <x:v>first_test_h_median_iqr</x:v>
+      </x:c>
+      <x:c r="G1" s="44" t="str">
+        <x:v>occasions_median_iqr</x:v>
+      </x:c>
+      <x:c r="H1" s="44" t="str">
+        <x:v>opportunity_h_median_iqr</x:v>
+      </x:c>
+      <x:c r="I1" s="44" t="str">
+        <x:v>late_test_n</x:v>
+      </x:c>
+      <x:c r="J1" s="44" t="str">
+        <x:v>late_test_pct</x:v>
+      </x:c>
+      <x:c r="K1" s="44" t="str">
+        <x:v>late_opportunity_n</x:v>
+      </x:c>
+      <x:c r="L1" s="44" t="str">
+        <x:v>late_among_opportunity_n</x:v>
+      </x:c>
+      <x:c r="M1" s="44" t="str">
+        <x:v>late_among_opportunity_pct</x:v>
+      </x:c>
+      <x:c r="N1" s="44" t="str">
+        <x:v>source_risk_min</x:v>
+      </x:c>
+      <x:c r="O1" s="44" t="str">
+        <x:v>source_risk_max</x:v>
+      </x:c>
+      <x:c r="P1" s="44" t="str">
+        <x:v>source_risk_median</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="36" customHeight="1">
+      <x:c r="A2" s="45" t="str">
+        <x:v>INSPIRE</x:v>
+      </x:c>
+      <x:c r="B2" s="45" t="str">
+        <x:v>Q1</x:v>
+      </x:c>
+      <x:c r="C2" s="45" t="n">
+        <x:v>6680</x:v>
+      </x:c>
+      <x:c r="D2" s="45" t="n">
+        <x:v>3092</x:v>
+      </x:c>
+      <x:c r="E2" s="46" t="n">
+        <x:v>46.2874251497006</x:v>
+      </x:c>
+      <x:c r="F2" s="45" t="str">
+        <x:v>13.5 (0.4-36.9)</x:v>
+      </x:c>
+      <x:c r="G2" s="45" t="str">
+        <x:v>2.0 (1.0-3.0)</x:v>
+      </x:c>
+      <x:c r="H2" s="45" t="str">
+        <x:v>59.8 (36.7-107.2)</x:v>
+      </x:c>
+      <x:c r="I2" s="45" t="n">
+        <x:v>1277</x:v>
+      </x:c>
+      <x:c r="J2" s="46" t="n">
+        <x:v>19.11676646706587</x:v>
+      </x:c>
+      <x:c r="K2" s="45" t="n">
+        <x:v>4244</x:v>
+      </x:c>
+      <x:c r="L2" s="45" t="n">
+        <x:v>1277</x:v>
+      </x:c>
+      <x:c r="M2" s="46" t="n">
+        <x:v>30.089538171536283</x:v>
+      </x:c>
+      <x:c r="N2" s="45" t="n">
+        <x:v>0.0100756237961561</x:v>
+      </x:c>
+      <x:c r="O2" s="45" t="n">
+        <x:v>0.0290507191886959</x:v>
+      </x:c>
+      <x:c r="P2" s="45" t="n">
+        <x:v>0.0241914793628104</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="36" customHeight="1">
+      <x:c r="A3" s="45" t="str">
+        <x:v>INSPIRE</x:v>
+      </x:c>
+      <x:c r="B3" s="45" t="str">
+        <x:v>Q2</x:v>
+      </x:c>
+      <x:c r="C3" s="45" t="n">
+        <x:v>6678</x:v>
+      </x:c>
+      <x:c r="D3" s="45" t="n">
+        <x:v>4147</x:v>
+      </x:c>
+      <x:c r="E3" s="46" t="n">
+        <x:v>62.099430967355495</x:v>
+      </x:c>
+      <x:c r="F3" s="45" t="str">
+        <x:v>1.7 (0.3-34.0)</x:v>
+      </x:c>
+      <x:c r="G3" s="45" t="str">
+        <x:v>2.0 (1.0-4.0)</x:v>
+      </x:c>
+      <x:c r="H3" s="45" t="str">
+        <x:v>97.6 (55.0-134.8)</x:v>
+      </x:c>
+      <x:c r="I3" s="45" t="n">
+        <x:v>2506</x:v>
+      </x:c>
+      <x:c r="J3" s="46" t="n">
+        <x:v>37.526205450733755</x:v>
+      </x:c>
+      <x:c r="K3" s="45" t="n">
+        <x:v>5192</x:v>
+      </x:c>
+      <x:c r="L3" s="45" t="n">
+        <x:v>2506</x:v>
+      </x:c>
+      <x:c r="M3" s="46" t="n">
+        <x:v>48.26656394453004</x:v>
+      </x:c>
+      <x:c r="N3" s="45" t="n">
+        <x:v>0.0290544487617087</x:v>
+      </x:c>
+      <x:c r="O3" s="45" t="n">
+        <x:v>0.0395265885604018</x:v>
+      </x:c>
+      <x:c r="P3" s="45" t="n">
+        <x:v>0.0341884715087134</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="36" customHeight="1">
+      <x:c r="A4" s="45" t="str">
+        <x:v>INSPIRE</x:v>
+      </x:c>
+      <x:c r="B4" s="45" t="str">
+        <x:v>Q3</x:v>
+      </x:c>
+      <x:c r="C4" s="45" t="n">
+        <x:v>6679</x:v>
+      </x:c>
+      <x:c r="D4" s="45" t="n">
+        <x:v>5349</x:v>
+      </x:c>
+      <x:c r="E4" s="46" t="n">
+        <x:v>80.08683934720766</x:v>
+      </x:c>
+      <x:c r="F4" s="45" t="str">
+        <x:v>0.6 (0.3-19.9)</x:v>
+      </x:c>
+      <x:c r="G4" s="45" t="str">
+        <x:v>3.0 (2.0-4.0)</x:v>
+      </x:c>
+      <x:c r="H4" s="45" t="str">
+        <x:v>127.8 (79.6-168.0)</x:v>
+      </x:c>
+      <x:c r="I4" s="45" t="n">
+        <x:v>3927</x:v>
+      </x:c>
+      <x:c r="J4" s="46" t="n">
+        <x:v>58.79622698008684</x:v>
+      </x:c>
+      <x:c r="K4" s="45" t="n">
+        <x:v>5903</x:v>
+      </x:c>
+      <x:c r="L4" s="45" t="n">
+        <x:v>3927</x:v>
+      </x:c>
+      <x:c r="M4" s="46" t="n">
+        <x:v>66.52549551075724</x:v>
+      </x:c>
+      <x:c r="N4" s="45" t="n">
+        <x:v>0.0395276806339759</x:v>
+      </x:c>
+      <x:c r="O4" s="45" t="n">
+        <x:v>0.0533838856963738</x:v>
+      </x:c>
+      <x:c r="P4" s="45" t="n">
+        <x:v>0.0456680020760114</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="36" customHeight="1">
+      <x:c r="A5" s="45" t="str">
+        <x:v>INSPIRE</x:v>
+      </x:c>
+      <x:c r="B5" s="45" t="str">
+        <x:v>Q4</x:v>
+      </x:c>
+      <x:c r="C5" s="45" t="n">
+        <x:v>6678</x:v>
+      </x:c>
+      <x:c r="D5" s="45" t="n">
+        <x:v>6001</x:v>
+      </x:c>
+      <x:c r="E5" s="46" t="n">
+        <x:v>89.86223420185684</x:v>
+      </x:c>
+      <x:c r="F5" s="45" t="str">
+        <x:v>0.5 (0.2-2.9)</x:v>
+      </x:c>
+      <x:c r="G5" s="45" t="str">
+        <x:v>4.0 (3.0-5.0)</x:v>
+      </x:c>
+      <x:c r="H5" s="45" t="str">
+        <x:v>168.0 (108.4-168.0)</x:v>
+      </x:c>
+      <x:c r="I5" s="45" t="n">
+        <x:v>5157</x:v>
+      </x:c>
+      <x:c r="J5" s="46" t="n">
+        <x:v>77.22371967654986</x:v>
+      </x:c>
+      <x:c r="K5" s="45" t="n">
+        <x:v>6338</x:v>
+      </x:c>
+      <x:c r="L5" s="45" t="n">
+        <x:v>5157</x:v>
+      </x:c>
+      <x:c r="M5" s="46" t="n">
+        <x:v>81.3663616282739</x:v>
+      </x:c>
+      <x:c r="N5" s="45" t="n">
+        <x:v>0.0533874060632093</x:v>
+      </x:c>
+      <x:c r="O5" s="45" t="n">
+        <x:v>0.0773548156758252</x:v>
+      </x:c>
+      <x:c r="P5" s="45" t="n">
+        <x:v>0.0633895471097351</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="36" customHeight="1">
+      <x:c r="A6" s="45" t="str">
+        <x:v>INSPIRE</x:v>
+      </x:c>
+      <x:c r="B6" s="45" t="str">
+        <x:v>Q5</x:v>
+      </x:c>
+      <x:c r="C6" s="45" t="n">
+        <x:v>6679</x:v>
+      </x:c>
+      <x:c r="D6" s="45" t="n">
+        <x:v>6283</x:v>
+      </x:c>
+      <x:c r="E6" s="46" t="n">
+        <x:v>94.0709687078904</x:v>
+      </x:c>
+      <x:c r="F6" s="45" t="str">
+        <x:v>0.5 (0.3-1.1)</x:v>
+      </x:c>
+      <x:c r="G6" s="45" t="str">
+        <x:v>5.0 (3.0-6.0)</x:v>
+      </x:c>
+      <x:c r="H6" s="45" t="str">
+        <x:v>168.0 (132.0-168.0)</x:v>
+      </x:c>
+      <x:c r="I6" s="45" t="n">
+        <x:v>5631</x:v>
+      </x:c>
+      <x:c r="J6" s="46" t="n">
+        <x:v>84.30902829764935</x:v>
+      </x:c>
+      <x:c r="K6" s="45" t="n">
+        <x:v>6389</x:v>
+      </x:c>
+      <x:c r="L6" s="45" t="n">
+        <x:v>5631</x:v>
+      </x:c>
+      <x:c r="M6" s="46" t="n">
+        <x:v>88.13585850680857</x:v>
+      </x:c>
+      <x:c r="N6" s="45" t="n">
+        <x:v>0.0773603100985055</x:v>
+      </x:c>
+      <x:c r="O6" s="45" t="n">
+        <x:v>0.4905202777474402</x:v>
+      </x:c>
+      <x:c r="P6" s="45" t="n">
+        <x:v>0.100390024502758</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="36" customHeight="1">
+      <x:c r="A7" s="45" t="str">
+        <x:v>MOVER 2021</x:v>
+      </x:c>
+      <x:c r="B7" s="45" t="str">
+        <x:v>Q1</x:v>
+      </x:c>
+      <x:c r="C7" s="45" t="n">
+        <x:v>561</x:v>
+      </x:c>
+      <x:c r="D7" s="45" t="n">
+        <x:v>352</x:v>
+      </x:c>
+      <x:c r="E7" s="46" t="n">
+        <x:v>62.74509803921568</x:v>
+      </x:c>
+      <x:c r="F7" s="45" t="str">
+        <x:v>14.8 (10.4-18.5)</x:v>
+      </x:c>
+      <x:c r="G7" s="45" t="str">
+        <x:v>2.0 (1.0-6.0)</x:v>
+      </x:c>
+      <x:c r="H7" s="45" t="str">
+        <x:v>26.7 (8.0-81.5)</x:v>
+      </x:c>
+      <x:c r="I7" s="45" t="n">
+        <x:v>155</x:v>
+      </x:c>
+      <x:c r="J7" s="46" t="n">
+        <x:v>27.629233511586452</x:v>
+      </x:c>
+      <x:c r="K7" s="45" t="n">
+        <x:v>208</x:v>
+      </x:c>
+      <x:c r="L7" s="45" t="n">
+        <x:v>155</x:v>
+      </x:c>
+      <x:c r="M7" s="46" t="n">
+        <x:v>74.51923076923077</x:v>
+      </x:c>
+      <x:c r="N7" s="45" t="n">
+        <x:v>0.013229173846128</x:v>
+      </x:c>
+      <x:c r="O7" s="45" t="n">
+        <x:v>0.0348095363041429</x:v>
+      </x:c>
+      <x:c r="P7" s="45" t="n">
+        <x:v>0.0281031008803303</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="36" customHeight="1">
+      <x:c r="A8" s="45" t="str">
+        <x:v>MOVER 2021</x:v>
+      </x:c>
+      <x:c r="B8" s="45" t="str">
+        <x:v>Q2</x:v>
+      </x:c>
+      <x:c r="C8" s="45" t="n">
+        <x:v>560</x:v>
+      </x:c>
+      <x:c r="D8" s="45" t="n">
+        <x:v>421</x:v>
+      </x:c>
+      <x:c r="E8" s="46" t="n">
+        <x:v>75.17857142857143</x:v>
+      </x:c>
+      <x:c r="F8" s="45" t="str">
+        <x:v>14.1 (5.8-18.8)</x:v>
+      </x:c>
+      <x:c r="G8" s="45" t="str">
+        <x:v>3.0 (1.0-6.0)</x:v>
+      </x:c>
+      <x:c r="H8" s="45" t="str">
+        <x:v>51.8 (20.8-123.5)</x:v>
+      </x:c>
+      <x:c r="I8" s="45" t="n">
+        <x:v>244</x:v>
+      </x:c>
+      <x:c r="J8" s="46" t="n">
+        <x:v>43.57142857142857</x:v>
+      </x:c>
+      <x:c r="K8" s="45" t="n">
+        <x:v>304</x:v>
+      </x:c>
+      <x:c r="L8" s="45" t="n">
+        <x:v>244</x:v>
+      </x:c>
+      <x:c r="M8" s="46" t="n">
+        <x:v>80.26315789473685</x:v>
+      </x:c>
+      <x:c r="N8" s="45" t="n">
+        <x:v>0.0348101958269405</x:v>
+      </x:c>
+      <x:c r="O8" s="45" t="n">
+        <x:v>0.0473511350641941</x:v>
+      </x:c>
+      <x:c r="P8" s="45" t="n">
+        <x:v>0.0411183228784417</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="36" customHeight="1">
+      <x:c r="A9" s="45" t="str">
+        <x:v>MOVER 2021</x:v>
+      </x:c>
+      <x:c r="B9" s="45" t="str">
+        <x:v>Q3</x:v>
+      </x:c>
+      <x:c r="C9" s="45" t="n">
+        <x:v>560</x:v>
+      </x:c>
+      <x:c r="D9" s="45" t="n">
+        <x:v>452</x:v>
+      </x:c>
+      <x:c r="E9" s="46" t="n">
+        <x:v>80.71428571428572</x:v>
+      </x:c>
+      <x:c r="F9" s="45" t="str">
+        <x:v>11.9 (2.2-16.4)</x:v>
+      </x:c>
+      <x:c r="G9" s="45" t="str">
+        <x:v>4.0 (2.0-7.0)</x:v>
+      </x:c>
+      <x:c r="H9" s="45" t="str">
+        <x:v>72.0 (24.2-153.6)</x:v>
+      </x:c>
+      <x:c r="I9" s="45" t="n">
+        <x:v>274</x:v>
+      </x:c>
+      <x:c r="J9" s="46" t="n">
+        <x:v>48.92857142857142</x:v>
+      </x:c>
+      <x:c r="K9" s="45" t="n">
+        <x:v>335</x:v>
+      </x:c>
+      <x:c r="L9" s="45" t="n">
+        <x:v>274</x:v>
+      </x:c>
+      <x:c r="M9" s="46" t="n">
+        <x:v>81.7910447761194</x:v>
+      </x:c>
+      <x:c r="N9" s="45" t="n">
+        <x:v>0.0473710792624394</x:v>
+      </x:c>
+      <x:c r="O9" s="45" t="n">
+        <x:v>0.0629546882611362</x:v>
+      </x:c>
+      <x:c r="P9" s="45" t="n">
+        <x:v>0.0541763584000627</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="36" customHeight="1">
+      <x:c r="A10" s="45" t="str">
+        <x:v>MOVER 2021</x:v>
+      </x:c>
+      <x:c r="B10" s="45" t="str">
+        <x:v>Q4</x:v>
+      </x:c>
+      <x:c r="C10" s="45" t="n">
+        <x:v>560</x:v>
+      </x:c>
+      <x:c r="D10" s="45" t="n">
+        <x:v>487</x:v>
+      </x:c>
+      <x:c r="E10" s="46" t="n">
+        <x:v>86.96428571428572</x:v>
+      </x:c>
+      <x:c r="F10" s="45" t="str">
+        <x:v>11.2 (1.7-16.2)</x:v>
+      </x:c>
+      <x:c r="G10" s="45" t="str">
+        <x:v>4.0 (2.0-7.0)</x:v>
+      </x:c>
+      <x:c r="H10" s="45" t="str">
+        <x:v>90.5 (31.8-168.0)</x:v>
+      </x:c>
+      <x:c r="I10" s="45" t="n">
+        <x:v>316</x:v>
+      </x:c>
+      <x:c r="J10" s="46" t="n">
+        <x:v>56.42857142857143</x:v>
+      </x:c>
+      <x:c r="K10" s="45" t="n">
+        <x:v>380</x:v>
+      </x:c>
+      <x:c r="L10" s="45" t="n">
+        <x:v>316</x:v>
+      </x:c>
+      <x:c r="M10" s="46" t="n">
+        <x:v>83.15789473684211</x:v>
+      </x:c>
+      <x:c r="N10" s="45" t="n">
+        <x:v>0.0629887185180674</x:v>
+      </x:c>
+      <x:c r="O10" s="45" t="n">
+        <x:v>0.094516440159964</x:v>
+      </x:c>
+      <x:c r="P10" s="45" t="n">
+        <x:v>0.0745543110969903</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="36" customHeight="1">
+      <x:c r="A11" s="45" t="str">
+        <x:v>MOVER 2021</x:v>
+      </x:c>
+      <x:c r="B11" s="45" t="str">
+        <x:v>Q5</x:v>
+      </x:c>
+      <x:c r="C11" s="45" t="n">
+        <x:v>561</x:v>
+      </x:c>
+      <x:c r="D11" s="45" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="E11" s="46" t="n">
+        <x:v>89.12655971479501</x:v>
+      </x:c>
+      <x:c r="F11" s="45" t="str">
+        <x:v>4.2 (1.3-14.1)</x:v>
+      </x:c>
+      <x:c r="G11" s="45" t="str">
+        <x:v>6.0 (3.0-9.0)</x:v>
+      </x:c>
+      <x:c r="H11" s="45" t="str">
+        <x:v>103.8 (45.8-168.0)</x:v>
+      </x:c>
+      <x:c r="I11" s="45" t="n">
+        <x:v>369</x:v>
+      </x:c>
+      <x:c r="J11" s="46" t="n">
+        <x:v>65.77540106951871</x:v>
+      </x:c>
+      <x:c r="K11" s="45" t="n">
+        <x:v>413</x:v>
+      </x:c>
+      <x:c r="L11" s="45" t="n">
+        <x:v>369</x:v>
+      </x:c>
+      <x:c r="M11" s="46" t="n">
+        <x:v>89.34624697336562</x:v>
+      </x:c>
+      <x:c r="N11" s="45" t="n">
+        <x:v>0.0945239399664034</x:v>
+      </x:c>
+      <x:c r="O11" s="45" t="n">
+        <x:v>0.659208861132225</x:v>
+      </x:c>
+      <x:c r="P11" s="45" t="n">
+        <x:v>0.1364987084291481</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="36" customHeight="1">
+      <x:c r="A12" s="45" t="str">
+        <x:v>MOVER 2022</x:v>
+      </x:c>
+      <x:c r="B12" s="45" t="str">
+        <x:v>Q1</x:v>
+      </x:c>
+      <x:c r="C12" s="45" t="n">
+        <x:v>518</x:v>
+      </x:c>
+      <x:c r="D12" s="45" t="n">
+        <x:v>318</x:v>
+      </x:c>
+      <x:c r="E12" s="46" t="n">
+        <x:v>61.38996138996139</x:v>
+      </x:c>
+      <x:c r="F12" s="45" t="str">
+        <x:v>14.9 (9.4-18.8)</x:v>
+      </x:c>
+      <x:c r="G12" s="45" t="str">
+        <x:v>3.0 (1.0-6.0)</x:v>
+      </x:c>
+      <x:c r="H12" s="45" t="str">
+        <x:v>27.5 (8.9-97.0)</x:v>
+      </x:c>
+      <x:c r="I12" s="45" t="n">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="J12" s="46" t="n">
+        <x:v>32.818532818532816</x:v>
+      </x:c>
+      <x:c r="K12" s="45" t="n">
+        <x:v>217</x:v>
+      </x:c>
+      <x:c r="L12" s="45" t="n">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="M12" s="46" t="n">
+        <x:v>78.3410138248848</x:v>
+      </x:c>
+      <x:c r="N12" s="45" t="n">
+        <x:v>0.0119808142642697</x:v>
+      </x:c>
+      <x:c r="O12" s="45" t="n">
+        <x:v>0.0335709546556225</x:v>
+      </x:c>
+      <x:c r="P12" s="45" t="n">
+        <x:v>0.0276731074858726</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="36" customHeight="1">
+      <x:c r="A13" s="45" t="str">
+        <x:v>MOVER 2022</x:v>
+      </x:c>
+      <x:c r="B13" s="45" t="str">
+        <x:v>Q2</x:v>
+      </x:c>
+      <x:c r="C13" s="45" t="n">
+        <x:v>517</x:v>
+      </x:c>
+      <x:c r="D13" s="45" t="n">
+        <x:v>379</x:v>
+      </x:c>
+      <x:c r="E13" s="46" t="n">
+        <x:v>73.30754352030948</x:v>
+      </x:c>
+      <x:c r="F13" s="45" t="str">
+        <x:v>14.4 (8.4-18.3)</x:v>
+      </x:c>
+      <x:c r="G13" s="45" t="str">
+        <x:v>3.0 (1.0-6.0)</x:v>
+      </x:c>
+      <x:c r="H13" s="45" t="str">
+        <x:v>55.2 (21.4-126.7)</x:v>
+      </x:c>
+      <x:c r="I13" s="45" t="n">
+        <x:v>210</x:v>
+      </x:c>
+      <x:c r="J13" s="46" t="n">
+        <x:v>40.61895551257253</x:v>
+      </x:c>
+      <x:c r="K13" s="45" t="n">
+        <x:v>291</x:v>
+      </x:c>
+      <x:c r="L13" s="45" t="n">
+        <x:v>210</x:v>
+      </x:c>
+      <x:c r="M13" s="46" t="n">
+        <x:v>72.16494845360825</x:v>
+      </x:c>
+      <x:c r="N13" s="45" t="n">
+        <x:v>0.0335712260775453</x:v>
+      </x:c>
+      <x:c r="O13" s="45" t="n">
+        <x:v>0.0455802277007083</x:v>
+      </x:c>
+      <x:c r="P13" s="45" t="n">
+        <x:v>0.0397900842511013</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="36" customHeight="1">
+      <x:c r="A14" s="45" t="str">
+        <x:v>MOVER 2022</x:v>
+      </x:c>
+      <x:c r="B14" s="45" t="str">
+        <x:v>Q3</x:v>
+      </x:c>
+      <x:c r="C14" s="45" t="n">
+        <x:v>517</x:v>
+      </x:c>
+      <x:c r="D14" s="45" t="n">
+        <x:v>407</x:v>
+      </x:c>
+      <x:c r="E14" s="46" t="n">
+        <x:v>78.72340425531915</x:v>
+      </x:c>
+      <x:c r="F14" s="45" t="str">
+        <x:v>12.8 (2.1-18.1)</x:v>
+      </x:c>
+      <x:c r="G14" s="45" t="str">
+        <x:v>4.0 (2.0-7.0)</x:v>
+      </x:c>
+      <x:c r="H14" s="45" t="str">
+        <x:v>71.8 (25.0-164.1)</x:v>
+      </x:c>
+      <x:c r="I14" s="45" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="J14" s="46" t="n">
+        <x:v>48.35589941972921</x:v>
+      </x:c>
+      <x:c r="K14" s="45" t="n">
+        <x:v>315</x:v>
+      </x:c>
+      <x:c r="L14" s="45" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="M14" s="46" t="n">
+        <x:v>79.36507936507937</x:v>
+      </x:c>
+      <x:c r="N14" s="45" t="n">
+        <x:v>0.0455867066606969</x:v>
+      </x:c>
+      <x:c r="O14" s="45" t="n">
+        <x:v>0.0612642197998095</x:v>
+      </x:c>
+      <x:c r="P14" s="45" t="n">
+        <x:v>0.052751491717209</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="36" customHeight="1">
+      <x:c r="A15" s="45" t="str">
+        <x:v>MOVER 2022</x:v>
+      </x:c>
+      <x:c r="B15" s="45" t="str">
+        <x:v>Q4</x:v>
+      </x:c>
+      <x:c r="C15" s="45" t="n">
+        <x:v>517</x:v>
+      </x:c>
+      <x:c r="D15" s="45" t="n">
+        <x:v>453</x:v>
+      </x:c>
+      <x:c r="E15" s="46" t="n">
+        <x:v>87.62088974854933</x:v>
+      </x:c>
+      <x:c r="F15" s="45" t="str">
+        <x:v>10.4 (1.7-15.8)</x:v>
+      </x:c>
+      <x:c r="G15" s="45" t="str">
+        <x:v>4.0 (2.0-7.0)</x:v>
+      </x:c>
+      <x:c r="H15" s="45" t="str">
+        <x:v>100.5 (43.3-168.0)</x:v>
+      </x:c>
+      <x:c r="I15" s="45" t="n">
+        <x:v>308</x:v>
+      </x:c>
+      <x:c r="J15" s="46" t="n">
+        <x:v>59.57446808510638</x:v>
+      </x:c>
+      <x:c r="K15" s="45" t="n">
+        <x:v>366</x:v>
+      </x:c>
+      <x:c r="L15" s="45" t="n">
+        <x:v>308</x:v>
+      </x:c>
+      <x:c r="M15" s="46" t="n">
+        <x:v>84.15300546448088</x:v>
+      </x:c>
+      <x:c r="N15" s="45" t="n">
+        <x:v>0.0612999523081266</x:v>
+      </x:c>
+      <x:c r="O15" s="45" t="n">
+        <x:v>0.090588372466847</x:v>
+      </x:c>
+      <x:c r="P15" s="45" t="n">
+        <x:v>0.0719864949393461</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="36" customHeight="1">
+      <x:c r="A16" s="45" t="str">
+        <x:v>MOVER 2022</x:v>
+      </x:c>
+      <x:c r="B16" s="45" t="str">
+        <x:v>Q5</x:v>
+      </x:c>
+      <x:c r="C16" s="45" t="n">
+        <x:v>518</x:v>
+      </x:c>
+      <x:c r="D16" s="45" t="n">
+        <x:v>476</x:v>
+      </x:c>
+      <x:c r="E16" s="46" t="n">
+        <x:v>91.8918918918919</x:v>
+      </x:c>
+      <x:c r="F16" s="45" t="str">
+        <x:v>3.1 (1.1-13.3)</x:v>
+      </x:c>
+      <x:c r="G16" s="45" t="str">
+        <x:v>7.0 (3.0-10.0)</x:v>
+      </x:c>
+      <x:c r="H16" s="45" t="str">
+        <x:v>141.7 (65.5-168.0)</x:v>
+      </x:c>
+      <x:c r="I16" s="45" t="n">
+        <x:v>367</x:v>
+      </x:c>
+      <x:c r="J16" s="46" t="n">
+        <x:v>70.84942084942085</x:v>
+      </x:c>
+      <x:c r="K16" s="45" t="n">
+        <x:v>419</x:v>
+      </x:c>
+      <x:c r="L16" s="45" t="n">
+        <x:v>367</x:v>
+      </x:c>
+      <x:c r="M16" s="46" t="n">
+        <x:v>87.58949880668257</x:v>
+      </x:c>
+      <x:c r="N16" s="45" t="n">
+        <x:v>0.0906495682332592</x:v>
+      </x:c>
+      <x:c r="O16" s="45" t="n">
+        <x:v>0.6533695670187187</x:v>
+      </x:c>
+      <x:c r="P16" s="45" t="n">
+        <x:v>0.1325443920499002</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="20" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="20" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="20" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="20" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="72" customHeight="1">
+      <x:c r="A1" s="44" t="str">
+        <x:v>cohort</x:v>
+      </x:c>
+      <x:c r="B1" s="44" t="str">
+        <x:v>group</x:v>
+      </x:c>
+      <x:c r="C1" s="44" t="str">
+        <x:v>eligible_n</x:v>
+      </x:c>
+      <x:c r="D1" s="44" t="str">
+        <x:v>observed_n</x:v>
+      </x:c>
+      <x:c r="E1" s="44" t="str">
+        <x:v>observed_pct</x:v>
+      </x:c>
+      <x:c r="F1" s="44" t="str">
+        <x:v>first_test_h_median_iqr</x:v>
+      </x:c>
+      <x:c r="G1" s="44" t="str">
+        <x:v>occasions_median_iqr</x:v>
+      </x:c>
+      <x:c r="H1" s="44" t="str">
+        <x:v>opportunity_h_median_iqr</x:v>
+      </x:c>
+      <x:c r="I1" s="44" t="str">
+        <x:v>early_test_n</x:v>
+      </x:c>
+      <x:c r="J1" s="44" t="str">
+        <x:v>early_test_pct</x:v>
+      </x:c>
+      <x:c r="K1" s="44" t="str">
+        <x:v>late_test_n</x:v>
+      </x:c>
+      <x:c r="L1" s="44" t="str">
+        <x:v>late_test_pct</x:v>
+      </x:c>
+      <x:c r="M1" s="44" t="str">
+        <x:v>late_opportunity_n</x:v>
+      </x:c>
+      <x:c r="N1" s="44" t="str">
+        <x:v>late_among_opportunity_n</x:v>
+      </x:c>
+      <x:c r="O1" s="44" t="str">
+        <x:v>late_among_opportunity_pct</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="36" customHeight="1">
+      <x:c r="A2" s="45" t="str">
+        <x:v>INSPIRE</x:v>
+      </x:c>
+      <x:c r="B2" s="45" t="str">
+        <x:v>&lt;=48 h</x:v>
+      </x:c>
+      <x:c r="C2" s="45" t="n">
+        <x:v>5328</x:v>
+      </x:c>
+      <x:c r="D2" s="45" t="n">
+        <x:v>1503</x:v>
+      </x:c>
+      <x:c r="E2" s="46" t="n">
+        <x:v>28.209459459459456</x:v>
+      </x:c>
+      <x:c r="F2" s="45" t="str">
+        <x:v>0.4 (0.2-0.7)</x:v>
+      </x:c>
+      <x:c r="G2" s="45" t="str">
+        <x:v>1.0 (1.0-1.0)</x:v>
+      </x:c>
+      <x:c r="H2" s="45" t="str">
+        <x:v>34.3 (31.5-37.3)</x:v>
+      </x:c>
+      <x:c r="I2" s="45" t="n">
+        <x:v>1503</x:v>
+      </x:c>
+      <x:c r="J2" s="46" t="n">
+        <x:v>28.209459459459456</x:v>
+      </x:c>
+      <x:c r="K2" s="45" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L2" s="46" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M2" s="45" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N2" s="45" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O2" s="46"/>
+    </x:row>
+    <x:row r="3" ht="36" customHeight="1">
+      <x:c r="A3" s="45" t="str">
+        <x:v>INSPIRE</x:v>
+      </x:c>
+      <x:c r="B3" s="45" t="str">
+        <x:v>&gt;48 h</x:v>
+      </x:c>
+      <x:c r="C3" s="45" t="n">
+        <x:v>28066</x:v>
+      </x:c>
+      <x:c r="D3" s="45" t="n">
+        <x:v>23369</x:v>
+      </x:c>
+      <x:c r="E3" s="46" t="n">
+        <x:v>83.26444808665289</x:v>
+      </x:c>
+      <x:c r="F3" s="45" t="str">
+        <x:v>0.6 (0.3-18.5)</x:v>
+      </x:c>
+      <x:c r="G3" s="45" t="str">
+        <x:v>4.0 (2.0-5.0)</x:v>
+      </x:c>
+      <x:c r="H3" s="45" t="str">
+        <x:v>147.3 (100.1-168.0)</x:v>
+      </x:c>
+      <x:c r="I3" s="45" t="n">
+        <x:v>22985</x:v>
+      </x:c>
+      <x:c r="J3" s="46" t="n">
+        <x:v>81.89624456637925</x:v>
+      </x:c>
+      <x:c r="K3" s="45" t="n">
+        <x:v>18498</x:v>
+      </x:c>
+      <x:c r="L3" s="46" t="n">
+        <x:v>65.90892895318179</x:v>
+      </x:c>
+      <x:c r="M3" s="45" t="n">
+        <x:v>28066</x:v>
+      </x:c>
+      <x:c r="N3" s="45" t="n">
+        <x:v>18498</x:v>
+      </x:c>
+      <x:c r="O3" s="46" t="n">
+        <x:v>65.90892895318179</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="36" customHeight="1">
+      <x:c r="A4" s="45" t="str">
+        <x:v>MOVER 2021</x:v>
+      </x:c>
+      <x:c r="B4" s="45" t="str">
+        <x:v>&lt;=48 h</x:v>
+      </x:c>
+      <x:c r="C4" s="45" t="n">
+        <x:v>1162</x:v>
+      </x:c>
+      <x:c r="D4" s="45" t="n">
+        <x:v>604</x:v>
+      </x:c>
+      <x:c r="E4" s="46" t="n">
+        <x:v>51.97934595524957</x:v>
+      </x:c>
+      <x:c r="F4" s="45" t="str">
+        <x:v>13.9 (9.2-17.4)</x:v>
+      </x:c>
+      <x:c r="G4" s="45" t="str">
+        <x:v>1.0 (1.0-2.0)</x:v>
+      </x:c>
+      <x:c r="H4" s="45" t="str">
+        <x:v>19.8 (6.0-27.2)</x:v>
+      </x:c>
+      <x:c r="I4" s="45" t="n">
+        <x:v>604</x:v>
+      </x:c>
+      <x:c r="J4" s="46" t="n">
+        <x:v>51.97934595524957</x:v>
+      </x:c>
+      <x:c r="K4" s="45" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L4" s="46" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M4" s="45" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N4" s="45" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O4" s="46"/>
+    </x:row>
+    <x:row r="5" ht="36" customHeight="1">
+      <x:c r="A5" s="45" t="str">
+        <x:v>MOVER 2021</x:v>
+      </x:c>
+      <x:c r="B5" s="45" t="str">
+        <x:v>&gt;48 h</x:v>
+      </x:c>
+      <x:c r="C5" s="45" t="n">
+        <x:v>1640</x:v>
+      </x:c>
+      <x:c r="D5" s="45" t="n">
+        <x:v>1608</x:v>
+      </x:c>
+      <x:c r="E5" s="46" t="n">
+        <x:v>98.04878048780488</x:v>
+      </x:c>
+      <x:c r="F5" s="45" t="str">
+        <x:v>10.5 (1.7-16.6)</x:v>
+      </x:c>
+      <x:c r="G5" s="45" t="str">
+        <x:v>6.0 (3.0-8.0)</x:v>
+      </x:c>
+      <x:c r="H5" s="45" t="str">
+        <x:v>132.5 (82.3-168.0)</x:v>
+      </x:c>
+      <x:c r="I5" s="45" t="n">
+        <x:v>1590</x:v>
+      </x:c>
+      <x:c r="J5" s="46" t="n">
+        <x:v>96.95121951219512</x:v>
+      </x:c>
+      <x:c r="K5" s="45" t="n">
+        <x:v>1358</x:v>
+      </x:c>
+      <x:c r="L5" s="46" t="n">
+        <x:v>82.80487804878048</x:v>
+      </x:c>
+      <x:c r="M5" s="45" t="n">
+        <x:v>1640</x:v>
+      </x:c>
+      <x:c r="N5" s="45" t="n">
+        <x:v>1358</x:v>
+      </x:c>
+      <x:c r="O5" s="46" t="n">
+        <x:v>82.80487804878048</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="36" customHeight="1">
+      <x:c r="A6" s="45" t="str">
+        <x:v>MOVER 2022</x:v>
+      </x:c>
+      <x:c r="B6" s="45" t="str">
+        <x:v>&lt;=48 h</x:v>
+      </x:c>
+      <x:c r="C6" s="45" t="n">
+        <x:v>979</x:v>
+      </x:c>
+      <x:c r="D6" s="45" t="n">
+        <x:v>478</x:v>
+      </x:c>
+      <x:c r="E6" s="46" t="n">
+        <x:v>48.825331971399386</x:v>
+      </x:c>
+      <x:c r="F6" s="45" t="str">
+        <x:v>13.8 (9.4-17.3)</x:v>
+      </x:c>
+      <x:c r="G6" s="45" t="str">
+        <x:v>1.0 (1.0-2.0)</x:v>
+      </x:c>
+      <x:c r="H6" s="45" t="str">
+        <x:v>20.1 (5.1-26.9)</x:v>
+      </x:c>
+      <x:c r="I6" s="45" t="n">
+        <x:v>478</x:v>
+      </x:c>
+      <x:c r="J6" s="46" t="n">
+        <x:v>48.825331971399386</x:v>
+      </x:c>
+      <x:c r="K6" s="45" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L6" s="46" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M6" s="45" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N6" s="45" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O6" s="46"/>
+    </x:row>
+    <x:row r="7" ht="36" customHeight="1">
+      <x:c r="A7" s="45" t="str">
+        <x:v>MOVER 2022</x:v>
+      </x:c>
+      <x:c r="B7" s="45" t="str">
+        <x:v>&gt;48 h</x:v>
+      </x:c>
+      <x:c r="C7" s="45" t="n">
+        <x:v>1608</x:v>
+      </x:c>
+      <x:c r="D7" s="45" t="n">
+        <x:v>1555</x:v>
+      </x:c>
+      <x:c r="E7" s="46" t="n">
+        <x:v>96.70398009950247</x:v>
+      </x:c>
+      <x:c r="F7" s="45" t="str">
+        <x:v>10.4 (1.6-17.0)</x:v>
+      </x:c>
+      <x:c r="G7" s="45" t="str">
+        <x:v>6.0 (3.0-8.0)</x:v>
+      </x:c>
+      <x:c r="H7" s="45" t="str">
+        <x:v>143.7 (82.5-168.0)</x:v>
+      </x:c>
+      <x:c r="I7" s="45" t="n">
+        <x:v>1540</x:v>
+      </x:c>
+      <x:c r="J7" s="46" t="n">
+        <x:v>95.77114427860695</x:v>
+      </x:c>
+      <x:c r="K7" s="45" t="n">
+        <x:v>1305</x:v>
+      </x:c>
+      <x:c r="L7" s="46" t="n">
+        <x:v>81.15671641791045</x:v>
+      </x:c>
+      <x:c r="M7" s="45" t="n">
+        <x:v>1608</x:v>
+      </x:c>
+      <x:c r="N7" s="45" t="n">
+        <x:v>1305</x:v>
+      </x:c>
+      <x:c r="O7" s="46" t="n">
+        <x:v>81.15671641791045</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="20" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="20" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="72" customHeight="1">
+      <x:c r="A1" s="44" t="str">
+        <x:v>cohort</x:v>
+      </x:c>
+      <x:c r="B1" s="44" t="str">
+        <x:v>elapsed_day</x:v>
+      </x:c>
+      <x:c r="C1" s="44" t="str">
+        <x:v>window_hours</x:v>
+      </x:c>
+      <x:c r="D1" s="44" t="str">
+        <x:v>tested_n</x:v>
+      </x:c>
+      <x:c r="E1" s="44" t="str">
+        <x:v>all_eligible_n</x:v>
+      </x:c>
+      <x:c r="F1" s="44" t="str">
+        <x:v>any_opportunity_n</x:v>
+      </x:c>
+      <x:c r="G1" s="44" t="str">
+        <x:v>full_opportunity_n</x:v>
+      </x:c>
+      <x:c r="H1" s="44" t="str">
+        <x:v>tested_full_opportunity_n</x:v>
+      </x:c>
+      <x:c r="I1" s="44" t="str">
+        <x:v>all_eligible_pct</x:v>
+      </x:c>
+      <x:c r="J1" s="44" t="str">
+        <x:v>any_opportunity_pct</x:v>
+      </x:c>
+      <x:c r="K1" s="44" t="str">
+        <x:v>full_opportunity_pct</x:v>
+      </x:c>
+      <x:c r="L1" s="44" t="str">
+        <x:v>any_opportunity_ci_low</x:v>
+      </x:c>
+      <x:c r="M1" s="44" t="str">
+        <x:v>any_opportunity_ci_high</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="36" customHeight="1">
+      <x:c r="A2" s="45" t="str">
+        <x:v>INSPIRE</x:v>
+      </x:c>
+      <x:c r="B2" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C2" s="45" t="str">
+        <x:v>(0,24]</x:v>
+      </x:c>
+      <x:c r="D2" s="45" t="n">
+        <x:v>20112</x:v>
+      </x:c>
+      <x:c r="E2" s="45" t="n">
+        <x:v>33394</x:v>
+      </x:c>
+      <x:c r="F2" s="45" t="n">
+        <x:v>33394</x:v>
+      </x:c>
+      <x:c r="G2" s="45" t="n">
+        <x:v>33064</x:v>
+      </x:c>
+      <x:c r="H2" s="45" t="n">
+        <x:v>20086</x:v>
+      </x:c>
+      <x:c r="I2" s="46" t="n">
+        <x:v>60.226387973887526</x:v>
+      </x:c>
+      <x:c r="J2" s="46" t="n">
+        <x:v>60.226387973887526</x:v>
+      </x:c>
+      <x:c r="K2" s="46" t="n">
+        <x:v>60.74885071376724</x:v>
+      </x:c>
+      <x:c r="L2" s="46" t="n">
+        <x:v>59.70030648385291</x:v>
+      </x:c>
+      <x:c r="M2" s="46" t="n">
+        <x:v>60.75011696169026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="36" customHeight="1">
+      <x:c r="A3" s="45" t="str">
+        <x:v>INSPIRE</x:v>
+      </x:c>
+      <x:c r="B3" s="45" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C3" s="45" t="str">
+        <x:v>(24,48]</x:v>
+      </x:c>
+      <x:c r="D3" s="45" t="n">
+        <x:v>18004</x:v>
+      </x:c>
+      <x:c r="E3" s="45" t="n">
+        <x:v>33394</x:v>
+      </x:c>
+      <x:c r="F3" s="45" t="n">
+        <x:v>33060</x:v>
+      </x:c>
+      <x:c r="G3" s="45" t="n">
+        <x:v>28077</x:v>
+      </x:c>
+      <x:c r="H3" s="45" t="n">
+        <x:v>17978</x:v>
+      </x:c>
+      <x:c r="I3" s="46" t="n">
+        <x:v>53.91387674432533</x:v>
+      </x:c>
+      <x:c r="J3" s="46" t="n">
+        <x:v>54.45856019358742</x:v>
+      </x:c>
+      <x:c r="K3" s="46" t="n">
+        <x:v>64.03105744915767</x:v>
+      </x:c>
+      <x:c r="L3" s="46" t="n">
+        <x:v>53.92124763879167</x:v>
+      </x:c>
+      <x:c r="M3" s="46" t="n">
+        <x:v>54.99483672990328</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="36" customHeight="1">
+      <x:c r="A4" s="45" t="str">
+        <x:v>INSPIRE</x:v>
+      </x:c>
+      <x:c r="B4" s="45" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C4" s="45" t="str">
+        <x:v>(48,72]</x:v>
+      </x:c>
+      <x:c r="D4" s="45" t="n">
+        <x:v>8067</x:v>
+      </x:c>
+      <x:c r="E4" s="45" t="n">
+        <x:v>33394</x:v>
+      </x:c>
+      <x:c r="F4" s="45" t="n">
+        <x:v>28066</x:v>
+      </x:c>
+      <x:c r="G4" s="45" t="n">
+        <x:v>24308</x:v>
+      </x:c>
+      <x:c r="H4" s="45" t="n">
+        <x:v>8021</x:v>
+      </x:c>
+      <x:c r="I4" s="46" t="n">
+        <x:v>24.157034197760076</x:v>
+      </x:c>
+      <x:c r="J4" s="46" t="n">
+        <x:v>28.742963015748593</x:v>
+      </x:c>
+      <x:c r="K4" s="46" t="n">
+        <x:v>32.99736712193516</x:v>
+      </x:c>
+      <x:c r="L4" s="46" t="n">
+        <x:v>28.216435085825488</x:v>
+      </x:c>
+      <x:c r="M4" s="46" t="n">
+        <x:v>29.275309149692884</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="36" customHeight="1">
+      <x:c r="A5" s="45" t="str">
+        <x:v>INSPIRE</x:v>
+      </x:c>
+      <x:c r="B5" s="45" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C5" s="45" t="str">
+        <x:v>(72,96]</x:v>
+      </x:c>
+      <x:c r="D5" s="45" t="n">
+        <x:v>9356</x:v>
+      </x:c>
+      <x:c r="E5" s="45" t="n">
+        <x:v>33394</x:v>
+      </x:c>
+      <x:c r="F5" s="45" t="n">
+        <x:v>24304</x:v>
+      </x:c>
+      <x:c r="G5" s="45" t="n">
+        <x:v>21343</x:v>
+      </x:c>
+      <x:c r="H5" s="45" t="n">
+        <x:v>9317</x:v>
+      </x:c>
+      <x:c r="I5" s="46" t="n">
+        <x:v>28.017009043540757</x:v>
+      </x:c>
+      <x:c r="J5" s="46" t="n">
+        <x:v>38.495720868992755</x:v>
+      </x:c>
+      <x:c r="K5" s="46" t="n">
+        <x:v>43.65365693670056</x:v>
+      </x:c>
+      <x:c r="L5" s="46" t="n">
+        <x:v>37.88584284048284</x:v>
+      </x:c>
+      <x:c r="M5" s="46" t="n">
+        <x:v>39.10923502575525</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="36" customHeight="1">
+      <x:c r="A6" s="45" t="str">
+        <x:v>INSPIRE</x:v>
+      </x:c>
+      <x:c r="B6" s="45" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C6" s="45" t="str">
+        <x:v>(96,120]</x:v>
+      </x:c>
+      <x:c r="D6" s="45" t="n">
+        <x:v>9544</x:v>
+      </x:c>
+      <x:c r="E6" s="45" t="n">
+        <x:v>33394</x:v>
+      </x:c>
+      <x:c r="F6" s="45" t="n">
+        <x:v>21336</x:v>
+      </x:c>
+      <x:c r="G6" s="45" t="n">
+        <x:v>17784</x:v>
+      </x:c>
+      <x:c r="H6" s="45" t="n">
+        <x:v>9512</x:v>
+      </x:c>
+      <x:c r="I6" s="46" t="n">
+        <x:v>28.57998442834042</x:v>
+      </x:c>
+      <x:c r="J6" s="46" t="n">
+        <x:v>44.73190851143607</x:v>
+      </x:c>
+      <x:c r="K6" s="46" t="n">
+        <x:v>53.48627980206928</x:v>
+      </x:c>
+      <x:c r="L6" s="46" t="n">
+        <x:v>44.06574463816642</x:v>
+      </x:c>
+      <x:c r="M6" s="46" t="n">
+        <x:v>45.39996903951975</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="36" customHeight="1">
+      <x:c r="A7" s="45" t="str">
+        <x:v>INSPIRE</x:v>
+      </x:c>
+      <x:c r="B7" s="45" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C7" s="45" t="str">
+        <x:v>(120,144]</x:v>
+      </x:c>
+      <x:c r="D7" s="45" t="n">
+        <x:v>4894</x:v>
+      </x:c>
+      <x:c r="E7" s="45" t="n">
+        <x:v>33394</x:v>
+      </x:c>
+      <x:c r="F7" s="45" t="n">
+        <x:v>17777</x:v>
+      </x:c>
+      <x:c r="G7" s="45" t="n">
+        <x:v>14197</x:v>
+      </x:c>
+      <x:c r="H7" s="45" t="n">
+        <x:v>4862</x:v>
+      </x:c>
+      <x:c r="I7" s="46" t="n">
+        <x:v>14.655327304306162</x:v>
+      </x:c>
+      <x:c r="J7" s="46" t="n">
+        <x:v>27.529954435506554</x:v>
+      </x:c>
+      <x:c r="K7" s="46" t="n">
+        <x:v>34.2466718320772</x:v>
+      </x:c>
+      <x:c r="L7" s="46" t="n">
+        <x:v>26.878261971652616</x:v>
+      </x:c>
+      <x:c r="M7" s="46" t="n">
+        <x:v>28.191355973583455</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="36" customHeight="1">
+      <x:c r="A8" s="45" t="str">
+        <x:v>INSPIRE</x:v>
+      </x:c>
+      <x:c r="B8" s="45" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C8" s="45" t="str">
+        <x:v>(144,168]</x:v>
+      </x:c>
+      <x:c r="D8" s="45" t="n">
+        <x:v>7497</x:v>
+      </x:c>
+      <x:c r="E8" s="45" t="n">
+        <x:v>33394</x:v>
+      </x:c>
+      <x:c r="F8" s="45" t="n">
+        <x:v>14194</x:v>
+      </x:c>
+      <x:c r="G8" s="45" t="n">
+        <x:v>11979</x:v>
+      </x:c>
+      <x:c r="H8" s="45" t="n">
+        <x:v>7466</x:v>
+      </x:c>
+      <x:c r="I8" s="46" t="n">
+        <x:v>22.4501407438462</x:v>
+      </x:c>
+      <x:c r="J8" s="46" t="n">
+        <x:v>52.81809215161336</x:v>
+      </x:c>
+      <x:c r="K8" s="46" t="n">
+        <x:v>62.325736705902</x:v>
+      </x:c>
+      <x:c r="L8" s="46" t="n">
+        <x:v>51.99619153715501</x:v>
+      </x:c>
+      <x:c r="M8" s="46" t="n">
+        <x:v>53.63846780398719</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="36" customHeight="1">
+      <x:c r="A9" s="45" t="str">
+        <x:v>MOVER 2021</x:v>
+      </x:c>
+      <x:c r="B9" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C9" s="45" t="str">
+        <x:v>(0,24]</x:v>
+      </x:c>
+      <x:c r="D9" s="45" t="n">
+        <x:v>2135</x:v>
+      </x:c>
+      <x:c r="E9" s="45" t="n">
+        <x:v>2802</x:v>
+      </x:c>
+      <x:c r="F9" s="45" t="n">
+        <x:v>2802</x:v>
+      </x:c>
+      <x:c r="G9" s="45" t="n">
+        <x:v>2060</x:v>
+      </x:c>
+      <x:c r="H9" s="45" t="n">
+        <x:v>1898</x:v>
+      </x:c>
+      <x:c r="I9" s="46" t="n">
+        <x:v>76.19557458957887</x:v>
+      </x:c>
+      <x:c r="J9" s="46" t="n">
+        <x:v>76.19557458957887</x:v>
+      </x:c>
+      <x:c r="K9" s="46" t="n">
+        <x:v>92.13592233009707</x:v>
+      </x:c>
+      <x:c r="L9" s="46" t="n">
+        <x:v>74.58346911769223</x:v>
+      </x:c>
+      <x:c r="M9" s="46" t="n">
+        <x:v>77.73595168867813</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="36" customHeight="1">
+      <x:c r="A10" s="45" t="str">
+        <x:v>MOVER 2021</x:v>
+      </x:c>
+      <x:c r="B10" s="45" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C10" s="45" t="str">
+        <x:v>(24,48]</x:v>
+      </x:c>
+      <x:c r="D10" s="45" t="n">
+        <x:v>1594</x:v>
+      </x:c>
+      <x:c r="E10" s="45" t="n">
+        <x:v>2802</x:v>
+      </x:c>
+      <x:c r="F10" s="45" t="n">
+        <x:v>2060</x:v>
+      </x:c>
+      <x:c r="G10" s="45" t="n">
+        <x:v>1640</x:v>
+      </x:c>
+      <x:c r="H10" s="45" t="n">
+        <x:v>1454</x:v>
+      </x:c>
+      <x:c r="I10" s="46" t="n">
+        <x:v>56.887937187723054</x:v>
+      </x:c>
+      <x:c r="J10" s="46" t="n">
+        <x:v>77.37864077669903</x:v>
+      </x:c>
+      <x:c r="K10" s="46" t="n">
+        <x:v>88.65853658536585</x:v>
+      </x:c>
+      <x:c r="L10" s="46" t="n">
+        <x:v>75.52195040750048</x:v>
+      </x:c>
+      <x:c r="M10" s="46" t="n">
+        <x:v>79.13341060286287</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="36" customHeight="1">
+      <x:c r="A11" s="45" t="str">
+        <x:v>MOVER 2021</x:v>
+      </x:c>
+      <x:c r="B11" s="45" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C11" s="45" t="str">
+        <x:v>(48,72]</x:v>
+      </x:c>
+      <x:c r="D11" s="45" t="n">
+        <x:v>1272</x:v>
+      </x:c>
+      <x:c r="E11" s="45" t="n">
+        <x:v>2802</x:v>
+      </x:c>
+      <x:c r="F11" s="45" t="n">
+        <x:v>1640</x:v>
+      </x:c>
+      <x:c r="G11" s="45" t="n">
+        <x:v>1354</x:v>
+      </x:c>
+      <x:c r="H11" s="45" t="n">
+        <x:v>1164</x:v>
+      </x:c>
+      <x:c r="I11" s="46" t="n">
+        <x:v>45.396145610278374</x:v>
+      </x:c>
+      <x:c r="J11" s="46" t="n">
+        <x:v>77.5609756097561</x:v>
+      </x:c>
+      <x:c r="K11" s="46" t="n">
+        <x:v>85.9675036927622</x:v>
+      </x:c>
+      <x:c r="L11" s="46" t="n">
+        <x:v>75.47883867063877</x:v>
+      </x:c>
+      <x:c r="M11" s="46" t="n">
+        <x:v>79.5142992107076</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="36" customHeight="1">
+      <x:c r="A12" s="45" t="str">
+        <x:v>MOVER 2021</x:v>
+      </x:c>
+      <x:c r="B12" s="45" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C12" s="45" t="str">
+        <x:v>(72,96]</x:v>
+      </x:c>
+      <x:c r="D12" s="45" t="n">
+        <x:v>1023</x:v>
+      </x:c>
+      <x:c r="E12" s="45" t="n">
+        <x:v>2802</x:v>
+      </x:c>
+      <x:c r="F12" s="45" t="n">
+        <x:v>1353</x:v>
+      </x:c>
+      <x:c r="G12" s="45" t="n">
+        <x:v>1115</x:v>
+      </x:c>
+      <x:c r="H12" s="45" t="n">
+        <x:v>930</x:v>
+      </x:c>
+      <x:c r="I12" s="46" t="n">
+        <x:v>36.50963597430407</x:v>
+      </x:c>
+      <x:c r="J12" s="46" t="n">
+        <x:v>75.60975609756098</x:v>
+      </x:c>
+      <x:c r="K12" s="46" t="n">
+        <x:v>83.40807174887892</x:v>
+      </x:c>
+      <x:c r="L12" s="46" t="n">
+        <x:v>73.25113012565167</x:v>
+      </x:c>
+      <x:c r="M12" s="46" t="n">
+        <x:v>77.82337054610142</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="36" customHeight="1">
+      <x:c r="A13" s="45" t="str">
+        <x:v>MOVER 2021</x:v>
+      </x:c>
+      <x:c r="B13" s="45" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C13" s="45" t="str">
+        <x:v>(96,120]</x:v>
+      </x:c>
+      <x:c r="D13" s="45" t="n">
+        <x:v>841</x:v>
+      </x:c>
+      <x:c r="E13" s="45" t="n">
+        <x:v>2802</x:v>
+      </x:c>
+      <x:c r="F13" s="45" t="n">
+        <x:v>1115</x:v>
+      </x:c>
+      <x:c r="G13" s="45" t="n">
+        <x:v>910</x:v>
+      </x:c>
+      <x:c r="H13" s="45" t="n">
+        <x:v>775</x:v>
+      </x:c>
+      <x:c r="I13" s="46" t="n">
+        <x:v>30.01427551748751</x:v>
+      </x:c>
+      <x:c r="J13" s="46" t="n">
+        <x:v>75.42600896860986</x:v>
+      </x:c>
+      <x:c r="K13" s="46" t="n">
+        <x:v>85.16483516483517</x:v>
+      </x:c>
+      <x:c r="L13" s="46" t="n">
+        <x:v>72.81452024847646</x:v>
+      </x:c>
+      <x:c r="M13" s="46" t="n">
+        <x:v>77.86290107247117</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="36" customHeight="1">
+      <x:c r="A14" s="45" t="str">
+        <x:v>MOVER 2021</x:v>
+      </x:c>
+      <x:c r="B14" s="45" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C14" s="45" t="str">
+        <x:v>(120,144]</x:v>
+      </x:c>
+      <x:c r="D14" s="45" t="n">
+        <x:v>680</x:v>
+      </x:c>
+      <x:c r="E14" s="45" t="n">
+        <x:v>2802</x:v>
+      </x:c>
+      <x:c r="F14" s="45" t="n">
+        <x:v>910</x:v>
+      </x:c>
+      <x:c r="G14" s="45" t="n">
+        <x:v>763</x:v>
+      </x:c>
+      <x:c r="H14" s="45" t="n">
+        <x:v>632</x:v>
+      </x:c>
+      <x:c r="I14" s="46" t="n">
+        <x:v>24.26837972876517</x:v>
+      </x:c>
+      <x:c r="J14" s="46" t="n">
+        <x:v>74.72527472527473</x:v>
+      </x:c>
+      <x:c r="K14" s="46" t="n">
+        <x:v>82.83093053735256</x:v>
+      </x:c>
+      <x:c r="L14" s="46" t="n">
+        <x:v>71.80175544482009</x:v>
+      </x:c>
+      <x:c r="M14" s="46" t="n">
+        <x:v>77.44092178944786</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="36" customHeight="1">
+      <x:c r="A15" s="45" t="str">
+        <x:v>MOVER 2021</x:v>
+      </x:c>
+      <x:c r="B15" s="45" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C15" s="45" t="str">
+        <x:v>(144,168]</x:v>
+      </x:c>
+      <x:c r="D15" s="45" t="n">
+        <x:v>571</x:v>
+      </x:c>
+      <x:c r="E15" s="45" t="n">
+        <x:v>2802</x:v>
+      </x:c>
+      <x:c r="F15" s="45" t="n">
+        <x:v>763</x:v>
+      </x:c>
+      <x:c r="G15" s="45" t="n">
+        <x:v>653</x:v>
+      </x:c>
+      <x:c r="H15" s="45" t="n">
+        <x:v>530</x:v>
+      </x:c>
+      <x:c r="I15" s="46" t="n">
+        <x:v>20.378301213418982</x:v>
+      </x:c>
+      <x:c r="J15" s="46" t="n">
+        <x:v>74.83617300131061</x:v>
+      </x:c>
+      <x:c r="K15" s="46" t="n">
+        <x:v>81.16385911179174</x:v>
+      </x:c>
+      <x:c r="L15" s="46" t="n">
+        <x:v>71.63781685723963</x:v>
+      </x:c>
+      <x:c r="M15" s="46" t="n">
+        <x:v>77.78569769593207</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="36" customHeight="1">
+      <x:c r="A16" s="45" t="str">
+        <x:v>MOVER 2022</x:v>
+      </x:c>
+      <x:c r="B16" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C16" s="45" t="str">
+        <x:v>(0,24]</x:v>
+      </x:c>
+      <x:c r="D16" s="45" t="n">
+        <x:v>1967</x:v>
+      </x:c>
+      <x:c r="E16" s="45" t="n">
+        <x:v>2587</x:v>
+      </x:c>
+      <x:c r="F16" s="45" t="n">
+        <x:v>2587</x:v>
+      </x:c>
+      <x:c r="G16" s="45" t="n">
+        <x:v>1950</x:v>
+      </x:c>
+      <x:c r="H16" s="45" t="n">
+        <x:v>1770</x:v>
+      </x:c>
+      <x:c r="I16" s="46" t="n">
+        <x:v>76.03401623502126</x:v>
+      </x:c>
+      <x:c r="J16" s="46" t="n">
+        <x:v>76.03401623502126</x:v>
+      </x:c>
+      <x:c r="K16" s="46" t="n">
+        <x:v>90.76923076923076</x:v>
+      </x:c>
+      <x:c r="L16" s="46" t="n">
+        <x:v>74.35123682640794</x:v>
+      </x:c>
+      <x:c r="M16" s="46" t="n">
+        <x:v>77.6395940063336</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="36" customHeight="1">
+      <x:c r="A17" s="45" t="str">
+        <x:v>MOVER 2022</x:v>
+      </x:c>
+      <x:c r="B17" s="45" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C17" s="45" t="str">
+        <x:v>(24,48]</x:v>
+      </x:c>
+      <x:c r="D17" s="45" t="n">
+        <x:v>1517</x:v>
+      </x:c>
+      <x:c r="E17" s="45" t="n">
+        <x:v>2587</x:v>
+      </x:c>
+      <x:c r="F17" s="45" t="n">
+        <x:v>1950</x:v>
+      </x:c>
+      <x:c r="G17" s="45" t="n">
+        <x:v>1608</x:v>
+      </x:c>
+      <x:c r="H17" s="45" t="n">
+        <x:v>1410</x:v>
+      </x:c>
+      <x:c r="I17" s="46" t="n">
+        <x:v>58.639350599149594</x:v>
+      </x:c>
+      <x:c r="J17" s="46" t="n">
+        <x:v>77.7948717948718</x:v>
+      </x:c>
+      <x:c r="K17" s="46" t="n">
+        <x:v>87.68656716417911</x:v>
+      </x:c>
+      <x:c r="L17" s="46" t="n">
+        <x:v>75.8964980151687</x:v>
+      </x:c>
+      <x:c r="M17" s="46" t="n">
+        <x:v>79.58395026308024</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="36" customHeight="1">
+      <x:c r="A18" s="45" t="str">
+        <x:v>MOVER 2022</x:v>
+      </x:c>
+      <x:c r="B18" s="45" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C18" s="45" t="str">
+        <x:v>(48,72]</x:v>
+      </x:c>
+      <x:c r="D18" s="45" t="n">
+        <x:v>1244</x:v>
+      </x:c>
+      <x:c r="E18" s="45" t="n">
+        <x:v>2587</x:v>
+      </x:c>
+      <x:c r="F18" s="45" t="n">
+        <x:v>1608</x:v>
+      </x:c>
+      <x:c r="G18" s="45" t="n">
+        <x:v>1328</x:v>
+      </x:c>
+      <x:c r="H18" s="45" t="n">
+        <x:v>1146</x:v>
+      </x:c>
+      <x:c r="I18" s="46" t="n">
+        <x:v>48.08658678005412</x:v>
+      </x:c>
+      <x:c r="J18" s="46" t="n">
+        <x:v>77.363184079602</x:v>
+      </x:c>
+      <x:c r="K18" s="46" t="n">
+        <x:v>86.29518072289157</x:v>
+      </x:c>
+      <x:c r="L18" s="46" t="n">
+        <x:v>75.25396058751984</x:v>
+      </x:c>
+      <x:c r="M18" s="46" t="n">
+        <x:v>79.34197967597562</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="36" customHeight="1">
+      <x:c r="A19" s="45" t="str">
+        <x:v>MOVER 2022</x:v>
+      </x:c>
+      <x:c r="B19" s="45" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C19" s="45" t="str">
+        <x:v>(72,96]</x:v>
+      </x:c>
+      <x:c r="D19" s="45" t="n">
+        <x:v>991</x:v>
+      </x:c>
+      <x:c r="E19" s="45" t="n">
+        <x:v>2587</x:v>
+      </x:c>
+      <x:c r="F19" s="45" t="n">
+        <x:v>1328</x:v>
+      </x:c>
+      <x:c r="G19" s="45" t="n">
+        <x:v>1118</x:v>
+      </x:c>
+      <x:c r="H19" s="45" t="n">
+        <x:v>927</x:v>
+      </x:c>
+      <x:c r="I19" s="46" t="n">
+        <x:v>38.30691921144182</x:v>
+      </x:c>
+      <x:c r="J19" s="46" t="n">
+        <x:v>74.62349397590361</x:v>
+      </x:c>
+      <x:c r="K19" s="46" t="n">
+        <x:v>82.91592128801432</x:v>
+      </x:c>
+      <x:c r="L19" s="46" t="n">
+        <x:v>72.21430251323589</x:v>
+      </x:c>
+      <x:c r="M19" s="46" t="n">
+        <x:v>76.8906412973508</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="36" customHeight="1">
+      <x:c r="A20" s="45" t="str">
+        <x:v>MOVER 2022</x:v>
+      </x:c>
+      <x:c r="B20" s="45" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C20" s="45" t="str">
+        <x:v>(96,120]</x:v>
+      </x:c>
+      <x:c r="D20" s="45" t="n">
+        <x:v>852</x:v>
+      </x:c>
+      <x:c r="E20" s="45" t="n">
+        <x:v>2587</x:v>
+      </x:c>
+      <x:c r="F20" s="45" t="n">
+        <x:v>1118</x:v>
+      </x:c>
+      <x:c r="G20" s="45" t="n">
+        <x:v>947</x:v>
+      </x:c>
+      <x:c r="H20" s="45" t="n">
+        <x:v>806</x:v>
+      </x:c>
+      <x:c r="I20" s="46" t="n">
+        <x:v>32.933900270583685</x:v>
+      </x:c>
+      <x:c r="J20" s="46" t="n">
+        <x:v>76.20751341681574</x:v>
+      </x:c>
+      <x:c r="K20" s="46" t="n">
+        <x:v>85.11087645195354</x:v>
+      </x:c>
+      <x:c r="L20" s="46" t="n">
+        <x:v>73.62442596148821</x:v>
+      </x:c>
+      <x:c r="M20" s="46" t="n">
+        <x:v>78.61111903397102</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="36" customHeight="1">
+      <x:c r="A21" s="45" t="str">
+        <x:v>MOVER 2022</x:v>
+      </x:c>
+      <x:c r="B21" s="45" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C21" s="45" t="str">
+        <x:v>(120,144]</x:v>
+      </x:c>
+      <x:c r="D21" s="45" t="n">
+        <x:v>710</x:v>
+      </x:c>
+      <x:c r="E21" s="45" t="n">
+        <x:v>2587</x:v>
+      </x:c>
+      <x:c r="F21" s="45" t="n">
+        <x:v>947</x:v>
+      </x:c>
+      <x:c r="G21" s="45" t="n">
+        <x:v>803</x:v>
+      </x:c>
+      <x:c r="H21" s="45" t="n">
+        <x:v>659</x:v>
+      </x:c>
+      <x:c r="I21" s="46" t="n">
+        <x:v>27.44491689215307</x:v>
+      </x:c>
+      <x:c r="J21" s="46" t="n">
+        <x:v>74.97360084477296</x:v>
+      </x:c>
+      <x:c r="K21" s="46" t="n">
+        <x:v>82.06724782067248</x:v>
+      </x:c>
+      <x:c r="L21" s="46" t="n">
+        <x:v>72.11759674578475</x:v>
+      </x:c>
+      <x:c r="M21" s="46" t="n">
+        <x:v>77.62781513251625</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="36" customHeight="1">
+      <x:c r="A22" s="45" t="str">
+        <x:v>MOVER 2022</x:v>
+      </x:c>
+      <x:c r="B22" s="45" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C22" s="45" t="str">
+        <x:v>(144,168]</x:v>
+      </x:c>
+      <x:c r="D22" s="45" t="n">
+        <x:v>607</x:v>
+      </x:c>
+      <x:c r="E22" s="45" t="n">
+        <x:v>2587</x:v>
+      </x:c>
+      <x:c r="F22" s="45" t="n">
+        <x:v>802</x:v>
+      </x:c>
+      <x:c r="G22" s="45" t="n">
+        <x:v>689</x:v>
+      </x:c>
+      <x:c r="H22" s="45" t="n">
+        <x:v>560</x:v>
+      </x:c>
+      <x:c r="I22" s="46" t="n">
+        <x:v>23.46347120216467</x:v>
+      </x:c>
+      <x:c r="J22" s="46" t="n">
+        <x:v>75.6857855361596</x:v>
+      </x:c>
+      <x:c r="K22" s="46" t="n">
+        <x:v>81.27721335268505</x:v>
+      </x:c>
+      <x:c r="L22" s="46" t="n">
+        <x:v>72.59897807941483</x:v>
+      </x:c>
+      <x:c r="M22" s="46" t="n">
+        <x:v>78.52770391122635</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr>
@@ -19210,6 +21679,92 @@
         <x:v>0.0119 (0.0054 to 0.0198)</x:v>
       </x:c>
     </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="100" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="44" customHeight="1">
+      <x:c r="A1" s="44" t="str">
+        <x:v>Item</x:v>
+      </x:c>
+      <x:c r="B1" s="44" t="str">
+        <x:v>Definition</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="44" customHeight="1">
+      <x:c r="A2" s="45" t="str">
+        <x:v>Analysis</x:v>
+      </x:c>
+      <x:c r="B2" s="45" t="str">
+        <x:v>Post hoc descriptive diagnostic, 7 October 2026; original labels and predictions fixed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="44" customHeight="1">
+      <x:c r="A3" s="45" t="str">
+        <x:v>Time zero</x:v>
+      </x:c>
+      <x:c r="B3" s="45" t="str">
+        <x:v>Anesthesia completion; (0,48] and (48,168] h within original recorded follow-up</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="44" customHeight="1">
+      <x:c r="A4" s="45" t="str">
+        <x:v>Opportunity</x:v>
+      </x:c>
+      <x:c r="B4" s="45" t="str">
+        <x:v>Separate all-eligible, any-bin and full-bin denominators; no adequate-surveillance criterion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="44" customHeight="1">
+      <x:c r="A5" s="45" t="str">
+        <x:v>Risk strata</x:v>
+      </x:c>
+      <x:c r="B5" s="45" t="str">
+        <x:v>Within-cohort quintiles of the frozen unupdated source model; source scores are in-sample descriptions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="44" customHeight="1">
+      <x:c r="A6" s="45" t="str">
+        <x:v>Intervals</x:v>
+      </x:c>
+      <x:c r="B6" s="45" t="str">
+        <x:v>Wilson 95% intervals describe proportions conditional on the retained cohort and recorded measurement process</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="44" customHeight="1">
+      <x:c r="A7" s="45" t="str">
+        <x:v>Provenance</x:v>
+      </x:c>
+      <x:c r="B7" s="45" t="str">
+        <x:v>Corrected primary tables originated in v3.3.0. Timing Tables S28-S31 are first included in v3.4.0; see the GitHub release for the assigned version DOI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="44" customHeight="1">
+      <x:c r="A8" s="45" t="str">
+        <x:v>Small cells</x:v>
+      </x:c>
+      <x:c r="B8" s="45" t="str">
+        <x:v>Positive counts below five and linked percentages/intervals suppressed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="44" customHeight="1">
+      <x:c r="A9" s="45" t="str">
+        <x:v>Raw data</x:v>
+      </x:c>
+      <x:c r="B9" s="45" t="str">
+        <x:v>Obtain from original providers; patient-level records are not included</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="44" customHeight="1"/>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>